<commit_message>
listo para entrega final
</commit_message>
<xml_diff>
--- a/Docs/TablasDatos-Lab6.xlsx
+++ b/Docs/TablasDatos-Lab6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Universidad\2025-2\Asistencia\Laboratorios\Lab6\ISIS1225-Laboratorio-6\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pcryz\Downloads\EDA\laboratorios\Lab 6\Laboratorio6-G10\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD33DA02-4501-4B58-9D83-E0FFBD1B4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{416FAC81-D631-4F24-9481-6B4C9A3FC6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
+    <workbookView xWindow="7200" yWindow="1065" windowWidth="21600" windowHeight="11295" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Lab6" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,6 +115,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -169,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +210,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -455,7 +472,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -626,6 +643,18 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>817303.46</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>575631.57999999996</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="General">
+                  <c:v>558909.76</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="General">
+                  <c:v>549734.97</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -635,6 +664,18 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>34316.239999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28390.77</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28117.58</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="General">
+                  <c:v>28822.06</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -731,8 +772,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$11:$B$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>620450.30000000005</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>598120.15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>585340.80000000005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>579210.4</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -740,8 +793,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$C$11:$C$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>31250.45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>32890.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>34100.65</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35680.199999999997</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1079,7 +1144,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1299,6 +1364,18 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>817303.46</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>575631.57999999996</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="General">
+                  <c:v>558909.76</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="General">
+                  <c:v>549734.97</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1443,8 +1520,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$11:$B$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>620450.30000000005</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>598120.15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>585340.80000000005</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>579210.4</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2839,7 +2928,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+    <xdr:ext cx="8654143" cy="6272893"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -2872,7 +2961,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+    <xdr:ext cx="8654143" cy="6272893"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -3252,29 +3341,45 @@
       <c r="A3" s="8">
         <v>0.1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="7"/>
+      <c r="B3" s="5">
+        <v>817303.46</v>
+      </c>
+      <c r="C3" s="7">
+        <v>34316.239999999998</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>0.5</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="7"/>
+      <c r="B4" s="2">
+        <v>575631.57999999996</v>
+      </c>
+      <c r="C4" s="7">
+        <v>28390.77</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>0.7</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7"/>
+      <c r="B5" s="12">
+        <v>558909.76</v>
+      </c>
+      <c r="C5" s="7">
+        <v>28117.58</v>
+      </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10">
         <v>0.9</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7"/>
+      <c r="B6" s="12">
+        <v>549734.97</v>
+      </c>
+      <c r="C6" s="12">
+        <v>28822.06</v>
+      </c>
     </row>
     <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
@@ -3298,29 +3403,48 @@
       <c r="A11" s="2">
         <v>2</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="5"/>
+      <c r="B11" s="13">
+        <v>620450.30000000005</v>
+      </c>
+      <c r="C11" s="5">
+        <v>31250.45</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>4</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="13">
+        <v>598120.15</v>
+      </c>
+      <c r="C12" s="13">
+        <v>32890.1</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>6</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="B13" s="13">
+        <v>585340.80000000005</v>
+      </c>
+      <c r="C13" s="13">
+        <v>34100.65</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>8</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="13">
+        <v>579210.4</v>
+      </c>
+      <c r="C14" s="13">
+        <v>35680.199999999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="14"/>
     </row>
     <row r="23" ht="14.65" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -3337,14 +3461,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3597,21 +3719,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3636,9 +3757,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>